<commit_message>
Add STIX file exploration scripts and enhance STIX I/O utilities for layer mapping
</commit_message>
<xml_diff>
--- a/baseline_models/bergambacht_runs.xlsx
+++ b/baseline_models/bergambacht_runs.xlsx
@@ -509,22 +509,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,55 +541,60 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
+          <t>layer_s1</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
           <t>active_model</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>gamma_dry</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>gamma_wet</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Su_S</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Su_m</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>MC_phi</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>MC_c</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>MC_psi</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>su_table_key</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Layers</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>POP</t>
         </is>
@@ -607,19 +613,24 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>L 1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>MohrCoulombClassic</t>
         </is>
-      </c>
-      <c r="D2" t="n">
-        <v>20</v>
       </c>
       <c r="E2" t="n">
         <v>20</v>
       </c>
-      <c r="H2" t="n">
+      <c r="F2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I2" t="n">
         <v>38</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -636,29 +647,34 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>10.5</v>
+          <t>L 2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E3" t="n">
         <v>10.5</v>
       </c>
       <c r="F3" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G3" t="n">
         <v>0.36</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>0.8</v>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>SP 1</t>
-        </is>
-      </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>26.8</t>
+          <t>SP 1, SP 25</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>26.8, 26.8</t>
         </is>
       </c>
     </row>
@@ -675,29 +691,34 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>19.5</v>
+          <t>L 3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E4" t="n">
         <v>19.5</v>
       </c>
       <c r="F4" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G4" t="n">
         <v>0.31</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>0.8</v>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>SP 2</t>
-        </is>
-      </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>27.4</t>
+          <t>SP 2, SP 24</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>27.4, 27.4</t>
         </is>
       </c>
     </row>
@@ -714,29 +735,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>17.5</v>
+          <t>L 4</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E5" t="n">
         <v>17.5</v>
       </c>
       <c r="F5" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G5" t="n">
         <v>0.31</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>0.8</v>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>SP 3</t>
-        </is>
-      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>27.4</t>
+          <t>SP 3, SP 23</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>27.4, 27.4</t>
         </is>
       </c>
     </row>
@@ -753,29 +779,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>10.1</v>
+          <t>L 5, L 16</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E6" t="n">
         <v>10.1</v>
       </c>
       <c r="F6" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G6" t="n">
         <v>0.37</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>1</v>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>SP 4, SP 5</t>
-        </is>
-      </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>18.7, 18.7</t>
+          <t>SP 22, SP 4, SP 27, SP 5</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>18.7, 18.7, 18.7, 18.7</t>
         </is>
       </c>
     </row>
@@ -792,29 +823,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>12</v>
+          <t>L 9, L 6</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E7" t="n">
         <v>12</v>
       </c>
       <c r="F7" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" t="n">
         <v>0.36</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>1</v>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>SP 6, SP 7</t>
-        </is>
-      </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>13.9, 13.9</t>
+          <t>SP 26, SP 7, SP 6</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>13.9, 13.9, 13.9</t>
         </is>
       </c>
     </row>
@@ -831,27 +867,32 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>15</v>
+          <t>L 7</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E8" t="n">
         <v>15</v>
       </c>
       <c r="F8" t="n">
+        <v>15</v>
+      </c>
+      <c r="G8" t="n">
         <v>0.31</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>1</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>SP 8</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>18.2</t>
         </is>
@@ -870,27 +911,32 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>13</v>
+          <t>L 8</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E9" t="n">
         <v>13</v>
       </c>
       <c r="F9" t="n">
+        <v>13</v>
+      </c>
+      <c r="G9" t="n">
         <v>0.3</v>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>1</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>SP 9</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>18.2</t>
         </is>
@@ -909,27 +955,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>10.5</v>
+          <t>L 17, L 10</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E10" t="n">
         <v>10.5</v>
       </c>
       <c r="F10" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G10" t="n">
         <v>0.35</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>0.8</v>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>SP 10, SP 11</t>
-        </is>
-      </c>
       <c r="M10" t="inlineStr">
+        <is>
+          <t>SP 11, SP 10</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
         <is>
           <t>26.8, 26.8</t>
         </is>
@@ -948,27 +999,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>17.5</v>
+          <t>L 13, L 11</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E11" t="n">
         <v>17.5</v>
       </c>
       <c r="F11" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="G11" t="n">
         <v>0.31</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>0.8</v>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>SP 12, SP 13</t>
-        </is>
-      </c>
       <c r="M11" t="inlineStr">
+        <is>
+          <t>SP 13, SP 12</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>27.4, 27.4</t>
         </is>
@@ -987,27 +1043,32 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>19.5</v>
+          <t>L 12</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E12" t="n">
         <v>19.5</v>
       </c>
       <c r="F12" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G12" t="n">
         <v>0.31</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>0.8</v>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>SP 14</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>27.4</t>
         </is>
@@ -1026,27 +1087,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>12</v>
+          <t>L 14</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E13" t="n">
         <v>12</v>
       </c>
       <c r="F13" t="n">
+        <v>12</v>
+      </c>
+      <c r="G13" t="n">
         <v>0.36</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>1</v>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>SP 15</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>13.9</t>
         </is>
@@ -1065,29 +1131,34 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>10.1</v>
+          <t>L 15</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E14" t="n">
         <v>10.1</v>
       </c>
       <c r="F14" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G14" t="n">
         <v>0.37</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>1</v>
       </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>SP 16</t>
-        </is>
-      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>18.7</t>
+          <t>SP 16, SP 28</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>18.7, 18.7</t>
         </is>
       </c>
     </row>
@@ -1104,27 +1175,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>17.2</v>
+          <t>L 18</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E15" t="n">
         <v>17.2</v>
       </c>
       <c r="F15" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="G15" t="n">
         <v>0.31</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>1</v>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>SP 17</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>27.4</t>
         </is>
@@ -1143,27 +1219,32 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>17.2</v>
+          <t>L 19</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E16" t="n">
         <v>17.2</v>
       </c>
       <c r="F16" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="G16" t="n">
         <v>0.31</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>0.8</v>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>SP 18</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>27.4</t>
         </is>
@@ -1182,27 +1263,32 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>10.1</v>
+          <t>L 20</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E17" t="n">
         <v>10.1</v>
       </c>
       <c r="F17" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="G17" t="n">
         <v>0.37</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>1</v>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>SP 19</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>18.7</t>
         </is>
@@ -1221,29 +1307,34 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Su</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>18.8</v>
+          <t>L 21, L 24</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Su</t>
+        </is>
       </c>
       <c r="E18" t="n">
         <v>18.8</v>
       </c>
       <c r="F18" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G18" t="n">
         <v>0.33</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>1</v>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>SP 20, SP 21</t>
-        </is>
-      </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>50.0, 50.0</t>
+          <t>SP 29, SP 20, SP 21, SP 30</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>50.0, 50.0, 50.0, 50.0</t>
         </is>
       </c>
     </row>
@@ -1260,19 +1351,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>L 23, L 25, L 22</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
           <t>MohrCoulombClassic</t>
         </is>
-      </c>
-      <c r="D19" t="n">
-        <v>17.8</v>
       </c>
       <c r="E19" t="n">
         <v>17.8</v>
       </c>
-      <c r="H19" t="n">
+      <c r="F19" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="I19" t="n">
         <v>32</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1289,19 +1385,24 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>L 26</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
           <t>MohrCoulombClassic</t>
         </is>
-      </c>
-      <c r="D20" t="n">
-        <v>19</v>
       </c>
       <c r="E20" t="n">
         <v>19</v>
       </c>
-      <c r="H20" t="n">
+      <c r="F20" t="n">
+        <v>19</v>
+      </c>
+      <c r="I20" t="n">
         <v>44.4</v>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update STIX and Excel files for bergambacht, eemdijk, ijkdijk models
</commit_message>
<xml_diff>
--- a/baseline_models/bergambacht_runs.xlsx
+++ b/baseline_models/bergambacht_runs.xlsx
@@ -514,7 +514,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -647,7 +647,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>L 2</t>
+          <t>L 3, L 2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>L 3</t>
+          <t>L 7, L 6</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>L 4</t>
+          <t>L 12, L 11</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>L 5, L 16</t>
+          <t>L 16, L 15, L 26, L 27</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>L 9, L 6</t>
+          <t>L 25, L 24, L 17</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>L 7</t>
+          <t>L 20</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>L 8</t>
+          <t>L 21</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>L 17, L 10</t>
+          <t>L 5, L 4</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>L 13, L 11</t>
+          <t>L 13, L 9</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>L 12</t>
+          <t>L 8</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>L 14</t>
+          <t>L 18</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>L 15</t>
+          <t>L 23, L 22</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1175,7 +1175,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>L 18</t>
+          <t>L 10</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>L 19</t>
+          <t>L 14</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>L 20</t>
+          <t>L 19</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>L 21, L 24</t>
+          <t>L 28, L 29, L 33, L 32</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>L 23, L 25, L 22</t>
+          <t>L 31, L 34, L 30</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>L 26</t>
+          <t>L 35</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">

</xml_diff>

<commit_message>
Update bergambacht_runs.xlsx and refactor run_model.py for improved error handling and output management
</commit_message>
<xml_diff>
--- a/baseline_models/bergambacht_runs.xlsx
+++ b/baseline_models/bergambacht_runs.xlsx
@@ -509,23 +509,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:O20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -536,65 +537,70 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>simple_description</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>material_code</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>layer_s1</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>active_model</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>gamma_dry</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>gamma_wet</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Su_S</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Su_m</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>MC_phi</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>MC_c</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>MC_psi</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>su_table_key</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Layers</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>POP</t>
         </is>
@@ -606,31 +612,31 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Material_KZ</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>L 1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>MohrCoulombClassic</t>
         </is>
-      </c>
-      <c r="E2" t="n">
-        <v>20</v>
       </c>
       <c r="F2" t="n">
         <v>20</v>
       </c>
-      <c r="I2" t="n">
+      <c r="G2" t="n">
+        <v>20</v>
+      </c>
+      <c r="J2" t="n">
         <v>38</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -640,39 +646,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Material_BVN</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>L 3, L 2</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E3" t="n">
-        <v>10.5</v>
       </c>
       <c r="F3" t="n">
         <v>10.5</v>
       </c>
       <c r="G3" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H3" t="n">
         <v>0.36</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>0.8</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>SP 1, SP 25</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>26.8, 26.8</t>
         </is>
@@ -684,39 +690,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Material_GZAN</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>L 7, L 6</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E4" t="n">
-        <v>19.5</v>
       </c>
       <c r="F4" t="n">
         <v>19.5</v>
       </c>
       <c r="G4" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="H4" t="n">
         <v>0.31</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>0.8</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>SP 2, SP 24</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>27.4, 27.4</t>
         </is>
@@ -728,39 +734,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Material_GZTN</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>L 12, L 11</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E5" t="n">
-        <v>17.5</v>
       </c>
       <c r="F5" t="n">
         <v>17.5</v>
       </c>
       <c r="G5" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H5" t="n">
         <v>0.31</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>0.8</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>SP 3, SP 23</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>27.4, 27.4</t>
         </is>
@@ -772,39 +778,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Material_HVN</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>L 16, L 15, L 26, L 27</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E6" t="n">
-        <v>10.1</v>
       </c>
       <c r="F6" t="n">
         <v>10.1</v>
       </c>
       <c r="G6" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H6" t="n">
         <v>0.37</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>SP 22, SP 4, SP 27, SP 5</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>18.7, 18.7, 18.7, 18.7</t>
         </is>
@@ -816,39 +822,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Material_GLN</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>L 25, L 24, L 17</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E7" t="n">
-        <v>12</v>
       </c>
       <c r="F7" t="n">
         <v>12</v>
       </c>
       <c r="G7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H7" t="n">
         <v>0.36</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>1</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>SP 26, SP 7, SP 6</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>13.9, 13.9, 13.9</t>
         </is>
@@ -860,39 +866,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Material_GZWN</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>L 20</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E8" t="n">
-        <v>15</v>
       </c>
       <c r="F8" t="n">
         <v>15</v>
       </c>
       <c r="G8" t="n">
+        <v>15</v>
+      </c>
+      <c r="H8" t="n">
         <v>0.31</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>1</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>SP 8</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>18.2</t>
         </is>
@@ -904,39 +910,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Material_GKN</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>L 21</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E9" t="n">
-        <v>13</v>
       </c>
       <c r="F9" t="n">
         <v>13</v>
       </c>
       <c r="G9" t="n">
+        <v>13</v>
+      </c>
+      <c r="H9" t="n">
         <v>0.3</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>SP 9</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>18.2</t>
         </is>
@@ -948,39 +954,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Material_BVO</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>L 5, L 4</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E10" t="n">
-        <v>10.5</v>
       </c>
       <c r="F10" t="n">
         <v>10.5</v>
       </c>
       <c r="G10" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H10" t="n">
         <v>0.35</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>0.8</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>SP 11, SP 10</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>26.8, 26.8</t>
         </is>
@@ -992,39 +998,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Material_GZTO</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>L 13, L 9</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E11" t="n">
-        <v>17.5</v>
       </c>
       <c r="F11" t="n">
         <v>17.5</v>
       </c>
       <c r="G11" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H11" t="n">
         <v>0.31</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>0.8</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>SP 13, SP 12</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>27.4, 27.4</t>
         </is>
@@ -1036,39 +1042,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Material_GZAO</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>L 8</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E12" t="n">
-        <v>19.5</v>
       </c>
       <c r="F12" t="n">
         <v>19.5</v>
       </c>
       <c r="G12" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="H12" t="n">
         <v>0.31</v>
       </c>
-      <c r="H12" t="n">
+      <c r="I12" t="n">
         <v>0.8</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>SP 14</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>27.4</t>
         </is>
@@ -1080,39 +1086,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Material_GLO</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>L 18</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E13" t="n">
-        <v>12</v>
       </c>
       <c r="F13" t="n">
         <v>12</v>
       </c>
       <c r="G13" t="n">
+        <v>12</v>
+      </c>
+      <c r="H13" t="n">
         <v>0.36</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>1</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>SP 15</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>13.9</t>
         </is>
@@ -1124,39 +1130,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Material_HVT</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>L 23, L 22</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E14" t="n">
-        <v>10.1</v>
       </c>
       <c r="F14" t="n">
         <v>10.1</v>
       </c>
       <c r="G14" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H14" t="n">
         <v>0.37</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>1</v>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>SP 16, SP 28</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>18.7, 18.7</t>
         </is>
@@ -1168,39 +1174,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Material_GZWO</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>L 10</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E15" t="n">
-        <v>17.2</v>
       </c>
       <c r="F15" t="n">
         <v>17.2</v>
       </c>
       <c r="G15" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="H15" t="n">
         <v>0.31</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>1</v>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>SP 17</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>27.4</t>
         </is>
@@ -1212,39 +1218,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Material_GKZO</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>L 14</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E16" t="n">
-        <v>17.2</v>
       </c>
       <c r="F16" t="n">
         <v>17.2</v>
       </c>
       <c r="G16" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="H16" t="n">
         <v>0.31</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>0.8</v>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>SP 18</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>27.4</t>
         </is>
@@ -1256,39 +1262,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Material_HVO</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>L 19</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E17" t="n">
-        <v>10.1</v>
       </c>
       <c r="F17" t="n">
         <v>10.1</v>
       </c>
       <c r="G17" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="H17" t="n">
         <v>0.37</v>
       </c>
-      <c r="H17" t="n">
+      <c r="I17" t="n">
         <v>1</v>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>SP 19</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>18.7</t>
         </is>
@@ -1300,39 +1306,39 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Material_OB</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>L 28, L 29, L 33, L 32</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Su</t>
         </is>
-      </c>
-      <c r="E18" t="n">
-        <v>18.8</v>
       </c>
       <c r="F18" t="n">
         <v>18.8</v>
       </c>
       <c r="G18" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="H18" t="n">
         <v>0.33</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>1</v>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>SP 29, SP 20, SP 21, SP 30</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>50.0, 50.0, 50.0, 50.0</t>
         </is>
@@ -1344,31 +1350,31 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Material_OA</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>L 31, L 34, L 30</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>MohrCoulombClassic</t>
         </is>
-      </c>
-      <c r="E19" t="n">
-        <v>17.8</v>
       </c>
       <c r="F19" t="n">
         <v>17.8</v>
       </c>
-      <c r="I19" t="n">
+      <c r="G19" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="J19" t="n">
         <v>32</v>
       </c>
-      <c r="J19" t="n">
+      <c r="K19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1378,31 +1384,31 @@
           <t>baseline</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Material_ST</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>L 35</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>MohrCoulombClassic</t>
         </is>
-      </c>
-      <c r="E20" t="n">
-        <v>19</v>
       </c>
       <c r="F20" t="n">
         <v>19</v>
       </c>
-      <c r="I20" t="n">
+      <c r="G20" t="n">
+        <v>19</v>
+      </c>
+      <c r="J20" t="n">
         <v>44.4</v>
       </c>
-      <c r="J20" t="n">
+      <c r="K20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1453,35 +1459,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>model_name</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>FoS_upliftvan</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>bergambacht</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-04-22 16:30:38</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.853386325909259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor generate_template.py and run_model.py to standardize constraints handling; remove unused su_tables sheet from Excel output
</commit_message>
<xml_diff>
--- a/baseline_models/bergambacht_runs.xlsx
+++ b/baseline_models/bergambacht_runs.xlsx
@@ -9,8 +9,7 @@
   <sheets>
     <sheet name="runs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="materials" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="su_tables" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="results" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="results" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,11 +47,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00375623"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="007B3F00"/>
       </patternFill>
     </fill>
     <fill>
@@ -73,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -82,9 +76,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -452,13 +443,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,6 +471,11 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>constraints</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>run_upliftvan</t>
         </is>
       </c>
@@ -494,8 +491,15 @@
           <t>Original model, no modifications</t>
         </is>
       </c>
-      <c r="D2" t="b">
-        <v>1</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1423,68 +1427,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>su_table_key</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>file</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>model_name</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>constraints</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>FoS_upliftvan</t>
         </is>

</xml_diff>

<commit_message>
Refactor run_model.py to improve material description handling and streamline constraint stripping logic
</commit_message>
<xml_diff>
--- a/baseline_models/bergambacht_runs.xlsx
+++ b/baseline_models/bergambacht_runs.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="runs" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +11,7 @@
     <sheet name="results" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -28,8 +27,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -41,17 +42,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00375623"/>
+        <fgColor rgb="FF375623"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004A235A"/>
+        <fgColor rgb="FF4A235A"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,7 +81,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -493,7 +494,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>BOTH</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -521,10 +522,8 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="6" max="7"/>
+    <col width="8" customWidth="1" min="8" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
@@ -1427,41 +1426,170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>run_id</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>model_name</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>constraints</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>FoS_upliftvan</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>baseline_cons</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>bergambacht</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-04-27 15:09:17</t>
+        </is>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.853386325909259</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>baseline_nocons</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>bergambacht</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-04-27 15:09:23</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>baseline_cons</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>bergambacht</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-04-27 15:15:10</t>
+        </is>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.853386325909259</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>baseline_nocons</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>bergambacht</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-04-27 15:15:18</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.853386325909259</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>baseline_cons</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>bergambacht</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-04-27 15:18:51</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.853386325909259</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>baseline_nocons</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>bergambacht</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-04-27 15:19:01</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.853386325909259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>